<commit_message>
sep-17-pass: marinetraffic.org cross-check of the remaining 81 imos folded into roll-forward batch; combined workbook, report and summary refreshed
</commit_message>
<xml_diff>
--- a/batches/2026-09-17_0421ET_fix_delivery_rollforward/lng_carrier_fix.xlsx
+++ b/batches/2026-09-17_0421ET_fix_delivery_rollforward/lng_carrier_fix.xlsx
@@ -501,7 +501,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Backend had not moved since June 2026. Every on-order row with an IMO was looked up in shipvault (status / delivered date / yard no.) and vesselfinder (AIS-registered name, MMSI, year built). Delivered vessels move to active with their real name; delivery years are corrected to the actual year; undelivered 2026 rows that shipvault now schedules for 2027+ are rolled forward. The rows vesselfinder never answered (IP ban at ~150/323) were cross-checked on marinetraffic.org the same afternoon (95 IMOs, paced).</t>
+          <t>Backend had not moved since June 2026. Every on-order row with an IMO was looked up in shipvault (status / delivered date / yard no.) and vesselfinder (AIS-registered name, MMSI, year built). Delivered vessels move to active with their real name; delivery years are corrected to the actual year; undelivered 2026 rows that shipvault now schedules for 2027+ are rolled forward. The rows vesselfinder never answered (IP ban at ~150/323) were cross-checked on marinetraffic.org the same afternoon (all 176 IMOs, paced, in two runs).</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Rows corrected: 150   Refs checked: 454   Refs dropped/removed: 0</t>
+          <t>Rows corrected: 151   Refs checked: 473   Refs dropped/removed: 0</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT151"/>
+  <dimension ref="A1:AT152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23057,14 +23057,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D132" s="7" t="inlineStr">
+      <c r="D132" s="5" t="inlineStr">
         <is>
           <t>Al Nasraniya</t>
         </is>
       </c>
       <c r="E132" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/476659, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476659</t>
+          <t>https://www.shipvault.com/ships/476659, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476659, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-NASRANIYA/1069821/538011621</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr"/>
@@ -23225,14 +23225,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D133" s="7" t="inlineStr">
+      <c r="D133" s="5" t="inlineStr">
         <is>
           <t>Al Yousifiya</t>
         </is>
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/476660, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476660</t>
+          <t>https://www.shipvault.com/ships/476660, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476660, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-YOUSIFIYA/1069845/1</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr"/>
@@ -23393,14 +23393,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D134" s="7" t="inlineStr">
+      <c r="D134" s="5" t="inlineStr">
         <is>
           <t>Athba</t>
         </is>
       </c>
       <c r="E134" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/476661, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476661</t>
+          <t>https://www.shipvault.com/ships/476661, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476661, https://www.marinetraffic.org/ship-owner-manager-ism-data/ATHBA/1069869/1</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr"/>
@@ -23561,14 +23561,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D135" s="7" t="inlineStr">
+      <c r="D135" s="5" t="inlineStr">
         <is>
           <t>E Qab</t>
         </is>
       </c>
       <c r="E135" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/476662, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476662</t>
+          <t>https://www.shipvault.com/ships/476662, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476662, https://www.marinetraffic.org/ship-owner-manager-ism-data/E-QAB/1069871/1</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr"/>
@@ -23729,14 +23729,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D136" s="7" t="inlineStr">
+      <c r="D136" s="5" t="inlineStr">
         <is>
           <t>Ghash Sham</t>
         </is>
       </c>
       <c r="E136" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478215, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478215</t>
+          <t>https://www.shipvault.com/ships/478215, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478215, https://www.marinetraffic.org/ship-owner-manager-ism-data/GHASH-SHAM/1069895/1</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr"/>
@@ -23897,14 +23897,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D137" s="7" t="inlineStr">
+      <c r="D137" s="5" t="inlineStr">
         <is>
           <t>Al Egdah</t>
         </is>
       </c>
       <c r="E137" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478216, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478216</t>
+          <t>https://www.shipvault.com/ships/478216, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478216, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-EGDAH/1069924/1</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr"/>
@@ -24065,14 +24065,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D138" s="7" t="inlineStr">
+      <c r="D138" s="5" t="inlineStr">
         <is>
           <t>Al Khbaib</t>
         </is>
       </c>
       <c r="E138" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478217, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478217</t>
+          <t>https://www.shipvault.com/ships/478217, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478217, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-KHBAIB/1069936/1</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr"/>
@@ -24233,14 +24233,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D139" s="7" t="inlineStr">
+      <c r="D139" s="5" t="inlineStr">
         <is>
           <t>Khowzan</t>
         </is>
       </c>
       <c r="E139" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478218, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478218</t>
+          <t>https://www.shipvault.com/ships/478218, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478218, https://www.marinetraffic.org/ship-owner-manager-ism-data/KHOWZAN/1069948/1</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr"/>
@@ -24401,14 +24401,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D140" s="7" t="inlineStr">
+      <c r="D140" s="5" t="inlineStr">
         <is>
           <t>Al Ghafat</t>
         </is>
       </c>
       <c r="E140" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478219, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478219</t>
+          <t>https://www.shipvault.com/ships/478219, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478219, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-GHAFAT/1069950/1</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr"/>
@@ -24569,14 +24569,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D141" s="7" t="inlineStr">
+      <c r="D141" s="5" t="inlineStr">
         <is>
           <t>Al Sidriya</t>
         </is>
       </c>
       <c r="E141" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478220, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478220</t>
+          <t>https://www.shipvault.com/ships/478220, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478220, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-SIDRIYA/1069962/1</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr"/>
@@ -24737,14 +24737,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D142" s="7" t="inlineStr">
+      <c r="D142" s="5" t="inlineStr">
         <is>
           <t>Lekhraib</t>
         </is>
       </c>
       <c r="E142" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/479139, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479139</t>
+          <t>https://www.shipvault.com/ships/479139, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479139, https://www.marinetraffic.org/ship-owner-manager-ism-data/LEKHRAIB/1070727/477262100</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr"/>
@@ -24905,14 +24905,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D143" s="7" t="inlineStr">
+      <c r="D143" s="5" t="inlineStr">
         <is>
           <t>Ain Snan</t>
         </is>
       </c>
       <c r="E143" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478221, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478221</t>
+          <t>https://www.shipvault.com/ships/478221, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478221, https://www.marinetraffic.org/ship-owner-manager-ism-data/AIN-SNAN/1069974/1</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr"/>
@@ -25073,14 +25073,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D144" s="7" t="inlineStr">
+      <c r="D144" s="5" t="inlineStr">
         <is>
           <t>Al Wasmi</t>
         </is>
       </c>
       <c r="E144" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478222, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478222</t>
+          <t>https://www.shipvault.com/ships/478222, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478222, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-WASMI/1069986/1</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr"/>
@@ -25241,14 +25241,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D145" s="7" t="inlineStr">
+      <c r="D145" s="5" t="inlineStr">
         <is>
           <t>Wadi Al Askar</t>
         </is>
       </c>
       <c r="E145" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/479141, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479141</t>
+          <t>https://www.shipvault.com/ships/479141, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479141, https://www.marinetraffic.org/ship-owner-manager-ism-data/WADI-AL-ASKAR/1070739/1</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr"/>
@@ -25409,14 +25409,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D146" s="7" t="inlineStr">
+      <c r="D146" s="5" t="inlineStr">
         <is>
           <t>Al Shaheen</t>
         </is>
       </c>
       <c r="E146" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/479144, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479144</t>
+          <t>https://www.shipvault.com/ships/479144, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479144, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-SHAHEEN/1070741/1</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr"/>
@@ -25564,12 +25564,12 @@
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>150</t>
         </is>
       </c>
       <c r="B147" s="4" t="inlineStr">
         <is>
-          <t>1070820</t>
+          <t>1070806</t>
         </is>
       </c>
       <c r="C147" s="4" t="inlineStr">
@@ -25579,12 +25579,12 @@
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>Al Nouf</t>
+          <t>Libsayer</t>
         </is>
       </c>
       <c r="E147" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/479151, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479151</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/LIBSAYER/1070806/1</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr"/>
@@ -25592,7 +25592,7 @@
       <c r="H147" s="2" t="inlineStr"/>
       <c r="I147" s="4" t="inlineStr">
         <is>
-          <t>Hull 2706 (SHI)</t>
+          <t>Hull 2702 (SHI)</t>
         </is>
       </c>
       <c r="J147" s="4" t="inlineStr">
@@ -25732,12 +25732,12 @@
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>154</t>
         </is>
       </c>
       <c r="B148" s="4" t="inlineStr">
         <is>
-          <t>1049091</t>
+          <t>1070820</t>
         </is>
       </c>
       <c r="C148" s="4" t="inlineStr">
@@ -25745,14 +25745,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D148" s="7" t="inlineStr">
-        <is>
-          <t>Izghawa</t>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>Al Nouf</t>
         </is>
       </c>
       <c r="E148" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478320, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478320</t>
+          <t>https://www.shipvault.com/ships/479151, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479151, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-NOUF/1070820/1</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr"/>
@@ -25760,7 +25760,7 @@
       <c r="H148" s="2" t="inlineStr"/>
       <c r="I148" s="4" t="inlineStr">
         <is>
-          <t>Hull 3491 (HDHHI)</t>
+          <t>Hull 2706 (SHI)</t>
         </is>
       </c>
       <c r="J148" s="4" t="inlineStr">
@@ -25790,7 +25790,7 @@
       </c>
       <c r="O148" s="4" t="inlineStr">
         <is>
-          <t>Nakilat</t>
+          <t>CMES</t>
         </is>
       </c>
       <c r="P148" s="4" t="inlineStr">
@@ -25802,7 +25802,7 @@
       <c r="R148" s="2" t="inlineStr"/>
       <c r="S148" s="4" t="inlineStr">
         <is>
-          <t>HD Hyundai Heavy Industries</t>
+          <t>Samsung Heavy Industries</t>
         </is>
       </c>
       <c r="T148" s="4" t="inlineStr">
@@ -25817,22 +25817,22 @@
       </c>
       <c r="V148" s="4" t="inlineStr">
         <is>
-          <t>https://www.hd.com/en/main</t>
+          <t>https://www.samsungshi.com/En/Default.aspx</t>
         </is>
       </c>
       <c r="W148" s="4" t="inlineStr">
         <is>
-          <t>35.51613</t>
+          <t>34.89804</t>
         </is>
       </c>
       <c r="X148" s="4" t="inlineStr">
         <is>
-          <t>129.4383</t>
+          <t>128.6045</t>
         </is>
       </c>
       <c r="Y148" s="4" t="inlineStr">
         <is>
-          <t>GC8Q+M6 Ulsan</t>
+          <t>VJW3+QV Geoje-si, Gyeongsangnam-do</t>
         </is>
       </c>
       <c r="Z148" s="4" t="inlineStr">
@@ -25842,7 +25842,7 @@
       </c>
       <c r="AA148" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/HD+Hyundai+Heavy+Industries+Ulsan+Shipyard/data=!3m1!1e3!4m10!1m2!2m1!1sHD+Hyundai!3m6!1s0x3567ce56ebbfb645:0xd94a696f9fca5d90!8m2!3d35.5167468!4d129.4380269!15sCgpIRCBIeXVuZGFpkgEIc2hpcHlhcmTgAQA!16s%2Fg%2F1tfhd8y1?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/Samsung+Heavy+industries/data=!3m1!1e3!4m10!1m2!2m1!1ssamsung+heavy+industries!3m6!1s0x356ecd83691a8fb5:0xd4204e9a1bb0ef10!8m2!3d34.8969682!4d128.6046376!15sChhzYW1zdW5nIGhlYXZ5IGluZHVzdHJpZXOSAQhzaGlweWFyZOABAA!16s%2Fg%2F1tgcpry6?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
         </is>
       </c>
       <c r="AB148" s="4" t="inlineStr">
@@ -25900,12 +25900,12 @@
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>222</t>
         </is>
       </c>
       <c r="B149" s="4" t="inlineStr">
         <is>
-          <t>1049118</t>
+          <t>1049091</t>
         </is>
       </c>
       <c r="C149" s="4" t="inlineStr">
@@ -25913,14 +25913,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D149" s="7" t="inlineStr">
-        <is>
-          <t>Al Wa'ab</t>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>Izghawa</t>
         </is>
       </c>
       <c r="E149" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478321, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478321</t>
+          <t>https://www.shipvault.com/ships/478320, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478320, https://www.marinetraffic.org/ship-owner-manager-ism-data/IZGHAWA/1049091/1</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr"/>
@@ -25928,7 +25928,7 @@
       <c r="H149" s="2" t="inlineStr"/>
       <c r="I149" s="4" t="inlineStr">
         <is>
-          <t>Hull 3492 (HDHHI)</t>
+          <t>Hull 3491 (HDHHI)</t>
         </is>
       </c>
       <c r="J149" s="4" t="inlineStr">
@@ -26068,12 +26068,12 @@
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
         <is>
-          <t>508</t>
+          <t>223</t>
         </is>
       </c>
       <c r="B150" s="4" t="inlineStr">
         <is>
-          <t>1069194</t>
+          <t>1049118</t>
         </is>
       </c>
       <c r="C150" s="4" t="inlineStr">
@@ -26081,21 +26081,29 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D150" s="7" t="inlineStr">
-        <is>
-          <t>Prime Glory</t>
+      <c r="D150" s="5" t="inlineStr">
+        <is>
+          <t>Al Wa'ab</t>
         </is>
       </c>
       <c r="E150" s="6" t="inlineStr">
         <is>
-          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/PRIME-GLORY/1069194/1</t>
+          <t>https://www.shipvault.com/ships/478321, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478321, https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-WA'AB/1049118/1</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr"/>
       <c r="G150" s="2" t="inlineStr"/>
       <c r="H150" s="2" t="inlineStr"/>
-      <c r="I150" s="2" t="inlineStr"/>
-      <c r="J150" s="2" t="inlineStr"/>
+      <c r="I150" s="4" t="inlineStr">
+        <is>
+          <t>Hull 3492 (HDHHI)</t>
+        </is>
+      </c>
+      <c r="J150" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
+        </is>
+      </c>
       <c r="K150" s="4" t="inlineStr">
         <is>
           <t>on order</t>
@@ -26118,7 +26126,7 @@
       </c>
       <c r="O150" s="4" t="inlineStr">
         <is>
-          <t>COSCO</t>
+          <t>Nakilat</t>
         </is>
       </c>
       <c r="P150" s="4" t="inlineStr">
@@ -26130,7 +26138,7 @@
       <c r="R150" s="2" t="inlineStr"/>
       <c r="S150" s="4" t="inlineStr">
         <is>
-          <t>DSIC (Dalian Shipbuilding Industry Co)</t>
+          <t>HD Hyundai Heavy Industries</t>
         </is>
       </c>
       <c r="T150" s="4" t="inlineStr">
@@ -26140,27 +26148,27 @@
       </c>
       <c r="U150" s="4" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="V150" s="4" t="inlineStr">
         <is>
-          <t>http://www.dsic.cn/English/CorporateProfile/AboutUs/index.htm</t>
+          <t>https://www.hd.com/en/main</t>
         </is>
       </c>
       <c r="W150" s="4" t="inlineStr">
         <is>
-          <t>38.937861</t>
+          <t>35.51613</t>
         </is>
       </c>
       <c r="X150" s="4" t="inlineStr">
         <is>
-          <t>121.638613</t>
+          <t>129.4383</t>
         </is>
       </c>
       <c r="Y150" s="4" t="inlineStr">
         <is>
-          <t>WJMP+FX6, Binhai St, Xigang District, Dalian, Dalian, Liaoning, China, 116006</t>
+          <t>GC8Q+M6 Ulsan</t>
         </is>
       </c>
       <c r="Z150" s="4" t="inlineStr">
@@ -26170,12 +26178,12 @@
       </c>
       <c r="AA150" s="4" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/place/Dalian+Shipbuilding+Heavy+Industry+Co.,Ltd./@38.9301597,121.6171177,2740m/data=!3m1!1e3!4m15!1m7!2m6!1sDalian+Shipbuilding+Industry+Co!3m4!2s60.153931,+24.928542!4m2!1d24.9285418!2d60.1539309!3m6!1s0x3585f55b64d083c7:0x46a88d8ffb6405f2!8m2!3d38.9336592!4d121.6374032!15sCh9EYWxpYW4gU2hpcGJ1aWxkaW5nIEluZHVzdHJ5IENvkgEHY29tcGFueeABAA!16s%2Fg%2F1tf_qtz_?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+          <t>https://www.google.com/maps/place/HD+Hyundai+Heavy+Industries+Ulsan+Shipyard/data=!3m1!1e3!4m10!1m2!2m1!1sHD+Hyundai!3m6!1s0x3567ce56ebbfb645:0xd94a696f9fca5d90!8m2!3d35.5167468!4d129.4380269!15sCgpIRCBIeXVuZGFpkgEIc2hpcHlhcmTgAQA!16s%2Fg%2F1tfhd8y1?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
         </is>
       </c>
       <c r="AB150" s="4" t="inlineStr">
         <is>
-          <t>175000</t>
+          <t>174000</t>
         </is>
       </c>
       <c r="AC150" s="4" t="inlineStr">
@@ -26228,12 +26236,12 @@
     <row r="151">
       <c r="A151" s="4" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>508</t>
         </is>
       </c>
       <c r="B151" s="4" t="inlineStr">
         <is>
-          <t>1030557</t>
+          <t>1069194</t>
         </is>
       </c>
       <c r="C151" s="4" t="inlineStr">
@@ -26241,14 +26249,14 @@
           <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
         </is>
       </c>
-      <c r="D151" s="5" t="inlineStr">
-        <is>
-          <t>Friendship Venture</t>
+      <c r="D151" s="7" t="inlineStr">
+        <is>
+          <t>Prime Glory</t>
         </is>
       </c>
       <c r="E151" s="6" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/469427, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/469427, https://www.marinetraffic.org/ship-owner-manager-ism-data/FRIENDSHIP-VENTURE/1030557/636025371</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/PRIME-GLORY/1069194/1</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr"/>
@@ -26278,7 +26286,7 @@
       </c>
       <c r="O151" s="4" t="inlineStr">
         <is>
-          <t>Wah Kwong, China Gas, CSSC</t>
+          <t>COSCO</t>
         </is>
       </c>
       <c r="P151" s="4" t="inlineStr">
@@ -26384,6 +26392,166 @@
       <c r="AR151" s="2" t="inlineStr"/>
       <c r="AS151" s="2" t="inlineStr"/>
       <c r="AT151" s="2" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="4" t="inlineStr">
+        <is>
+          <t>509</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>1030557</t>
+        </is>
+      </c>
+      <c r="C152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
+        </is>
+      </c>
+      <c r="D152" s="5" t="inlineStr">
+        <is>
+          <t>Friendship Venture</t>
+        </is>
+      </c>
+      <c r="E152" s="6" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/469427, https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/469427, https://www.marinetraffic.org/ship-owner-manager-ism-data/FRIENDSHIP-VENTURE/1030557/636025371</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr"/>
+      <c r="G152" s="2" t="inlineStr"/>
+      <c r="H152" s="2" t="inlineStr"/>
+      <c r="I152" s="2" t="inlineStr"/>
+      <c r="J152" s="2" t="inlineStr"/>
+      <c r="K152" s="4" t="inlineStr">
+        <is>
+          <t>on order</t>
+        </is>
+      </c>
+      <c r="L152" s="4" t="inlineStr">
+        <is>
+          <t>GEM</t>
+        </is>
+      </c>
+      <c r="M152" s="4" t="inlineStr">
+        <is>
+          <t>12/31/2024</t>
+        </is>
+      </c>
+      <c r="N152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
+        </is>
+      </c>
+      <c r="O152" s="4" t="inlineStr">
+        <is>
+          <t>Wah Kwong, China Gas, CSSC</t>
+        </is>
+      </c>
+      <c r="P152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
+        </is>
+      </c>
+      <c r="Q152" s="2" t="inlineStr"/>
+      <c r="R152" s="2" t="inlineStr"/>
+      <c r="S152" s="4" t="inlineStr">
+        <is>
+          <t>DSIC (Dalian Shipbuilding Industry Co)</t>
+        </is>
+      </c>
+      <c r="T152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
+        </is>
+      </c>
+      <c r="U152" s="4" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="V152" s="4" t="inlineStr">
+        <is>
+          <t>http://www.dsic.cn/English/CorporateProfile/AboutUs/index.htm</t>
+        </is>
+      </c>
+      <c r="W152" s="4" t="inlineStr">
+        <is>
+          <t>38.937861</t>
+        </is>
+      </c>
+      <c r="X152" s="4" t="inlineStr">
+        <is>
+          <t>121.638613</t>
+        </is>
+      </c>
+      <c r="Y152" s="4" t="inlineStr">
+        <is>
+          <t>WJMP+FX6, Binhai St, Xigang District, Dalian, Dalian, Liaoning, China, 116006</t>
+        </is>
+      </c>
+      <c r="Z152" s="4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AA152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/place/Dalian+Shipbuilding+Heavy+Industry+Co.,Ltd./@38.9301597,121.6171177,2740m/data=!3m1!1e3!4m15!1m7!2m6!1sDalian+Shipbuilding+Industry+Co!3m4!2s60.153931,+24.928542!4m2!1d24.9285418!2d60.1539309!3m6!1s0x3585f55b64d083c7:0x46a88d8ffb6405f2!8m2!3d38.9336592!4d121.6374032!15sCh9EYWxpYW4gU2hpcGJ1aWxkaW5nIEluZHVzdHJ5IENvkgEHY29tcGFueeABAA!16s%2Fg%2F1tf_qtz_?entry=ttu&amp;g_ep=EgoyMDI1MTIwMi4wIKXMDSoASAFQAw%3D%3D</t>
+        </is>
+      </c>
+      <c r="AB152" s="4" t="inlineStr">
+        <is>
+          <t>175000</t>
+        </is>
+      </c>
+      <c r="AC152" s="4" t="inlineStr">
+        <is>
+          <t>cbm</t>
+        </is>
+      </c>
+      <c r="AD152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
+        </is>
+      </c>
+      <c r="AE152" s="2" t="inlineStr"/>
+      <c r="AF152" s="2" t="inlineStr"/>
+      <c r="AG152" s="2" t="inlineStr"/>
+      <c r="AH152" s="2" t="inlineStr"/>
+      <c r="AI152" s="4" t="inlineStr">
+        <is>
+          <t>X-DF</t>
+        </is>
+      </c>
+      <c r="AJ152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
+        </is>
+      </c>
+      <c r="AK152" s="4" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="AL152" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igu.org/igu-reports/2025-world-lng-report</t>
+        </is>
+      </c>
+      <c r="AM152" s="4" t="inlineStr">
+        <is>
+          <t>IGU</t>
+        </is>
+      </c>
+      <c r="AN152" s="2" t="inlineStr"/>
+      <c r="AO152" s="2" t="inlineStr"/>
+      <c r="AP152" s="2" t="inlineStr"/>
+      <c r="AQ152" s="2" t="inlineStr"/>
+      <c r="AR152" s="2" t="inlineStr"/>
+      <c r="AS152" s="2" t="inlineStr"/>
+      <c r="AT152" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26396,7 +26564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F455"/>
+  <dimension ref="A1:F474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -39715,7 +39883,7 @@
       </c>
       <c r="F416" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2585 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2585 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069821 as AL NASRANIYA (MMSI 538011621)</t>
         </is>
       </c>
     </row>
@@ -39747,14 +39915,14 @@
       </c>
       <c r="F417" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2585 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2585 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069821 as AL NASRANIYA (MMSI 538011621)</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>80</t>
         </is>
       </c>
       <c r="B418" s="2" t="inlineStr">
@@ -39764,22 +39932,22 @@
       </c>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>Al Yousifiya</t>
+          <t>Al Nasraniya</t>
         </is>
       </c>
       <c r="D418" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/476660</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-NASRANIYA/1069821/538011621</t>
         </is>
       </c>
       <c r="E418" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F418" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2586 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2585 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069821 as AL NASRANIYA (MMSI 538011621)</t>
         </is>
       </c>
     </row>
@@ -39801,24 +39969,24 @@
       </c>
       <c r="D419" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476660</t>
+          <t>https://www.shipvault.com/ships/476660</t>
         </is>
       </c>
       <c r="E419" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F419" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2586 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2586 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069845 as AL YOUSIFIYA</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B420" s="2" t="inlineStr">
@@ -39828,29 +39996,29 @@
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>Athba</t>
+          <t>Al Yousifiya</t>
         </is>
       </c>
       <c r="D420" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/476661</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476660</t>
         </is>
       </c>
       <c r="E420" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F420" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2587 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2586 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069845 as AL YOUSIFIYA</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B421" s="2" t="inlineStr">
@@ -39860,29 +40028,29 @@
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
-          <t>Athba</t>
+          <t>Al Yousifiya</t>
         </is>
       </c>
       <c r="D421" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476661</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-YOUSIFIYA/1069845/1</t>
         </is>
       </c>
       <c r="E421" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F421" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2587 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2586 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069845 as AL YOUSIFIYA</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B422" s="2" t="inlineStr">
@@ -39892,12 +40060,12 @@
       </c>
       <c r="C422" s="2" t="inlineStr">
         <is>
-          <t>E Qab</t>
+          <t>Athba</t>
         </is>
       </c>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/476662</t>
+          <t>https://www.shipvault.com/ships/476661</t>
         </is>
       </c>
       <c r="E422" s="2" t="inlineStr">
@@ -39907,14 +40075,14 @@
       </c>
       <c r="F422" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2588 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2587 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069869 as ATHBA</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B423" s="2" t="inlineStr">
@@ -39924,12 +40092,12 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>E Qab</t>
+          <t>Athba</t>
         </is>
       </c>
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476662</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476661</t>
         </is>
       </c>
       <c r="E423" s="2" t="inlineStr">
@@ -39939,14 +40107,14 @@
       </c>
       <c r="F423" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2588 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2587 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069869 as ATHBA</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B424" s="2" t="inlineStr">
@@ -39956,29 +40124,29 @@
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>Ghash Sham</t>
+          <t>Athba</t>
         </is>
       </c>
       <c r="D424" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478215</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/ATHBA/1069869/1</t>
         </is>
       </c>
       <c r="E424" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F424" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2589 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2587 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069869 as ATHBA</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>83</t>
         </is>
       </c>
       <c r="B425" s="2" t="inlineStr">
@@ -39988,29 +40156,29 @@
       </c>
       <c r="C425" s="2" t="inlineStr">
         <is>
-          <t>Ghash Sham</t>
+          <t>E Qab</t>
         </is>
       </c>
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478215</t>
+          <t>https://www.shipvault.com/ships/476662</t>
         </is>
       </c>
       <c r="E425" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F425" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2589 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2588 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069871 as E QAB</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>83</t>
         </is>
       </c>
       <c r="B426" s="2" t="inlineStr">
@@ -40020,29 +40188,29 @@
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>Al Egdah</t>
+          <t>E Qab</t>
         </is>
       </c>
       <c r="D426" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478216</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/476662</t>
         </is>
       </c>
       <c r="E426" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F426" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2590 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2588 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069871 as E QAB</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>83</t>
         </is>
       </c>
       <c r="B427" s="2" t="inlineStr">
@@ -40052,29 +40220,29 @@
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>Al Egdah</t>
+          <t>E Qab</t>
         </is>
       </c>
       <c r="D427" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478216</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/E-QAB/1069871/1</t>
         </is>
       </c>
       <c r="E427" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F427" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2590 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2588 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069871 as E QAB</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B428" s="2" t="inlineStr">
@@ -40084,12 +40252,12 @@
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>Al Khbaib</t>
+          <t>Ghash Sham</t>
         </is>
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478217</t>
+          <t>https://www.shipvault.com/ships/478215</t>
         </is>
       </c>
       <c r="E428" s="2" t="inlineStr">
@@ -40099,14 +40267,14 @@
       </c>
       <c r="F428" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2591 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2589 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069895 as GHASH SHAM</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B429" s="2" t="inlineStr">
@@ -40116,12 +40284,12 @@
       </c>
       <c r="C429" s="2" t="inlineStr">
         <is>
-          <t>Al Khbaib</t>
+          <t>Ghash Sham</t>
         </is>
       </c>
       <c r="D429" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478217</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478215</t>
         </is>
       </c>
       <c r="E429" s="2" t="inlineStr">
@@ -40131,14 +40299,14 @@
       </c>
       <c r="F429" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2591 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2589 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069895 as GHASH SHAM</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B430" s="2" t="inlineStr">
@@ -40148,29 +40316,29 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>Khowzan</t>
+          <t>Ghash Sham</t>
         </is>
       </c>
       <c r="D430" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478218</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/GHASH-SHAM/1069895/1</t>
         </is>
       </c>
       <c r="E430" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F430" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2592 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2589 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069895 as GHASH SHAM</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B431" s="2" t="inlineStr">
@@ -40180,29 +40348,29 @@
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>Khowzan</t>
+          <t>Al Egdah</t>
         </is>
       </c>
       <c r="D431" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478218</t>
+          <t>https://www.shipvault.com/ships/478216</t>
         </is>
       </c>
       <c r="E431" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F431" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2592 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2590 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069924 as AL EGDAH</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B432" s="2" t="inlineStr">
@@ -40212,29 +40380,29 @@
       </c>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>Al Ghafat</t>
+          <t>Al Egdah</t>
         </is>
       </c>
       <c r="D432" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478219</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478216</t>
         </is>
       </c>
       <c r="E432" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F432" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2693 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2590 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069924 as AL EGDAH</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="inlineStr">
         <is>
-          <t>136</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B433" s="2" t="inlineStr">
@@ -40244,29 +40412,29 @@
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
-          <t>Al Ghafat</t>
+          <t>Al Egdah</t>
         </is>
       </c>
       <c r="D433" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478219</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-EGDAH/1069924/1</t>
         </is>
       </c>
       <c r="E433" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F433" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2693 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2590 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069924 as AL EGDAH</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>86</t>
         </is>
       </c>
       <c r="B434" s="2" t="inlineStr">
@@ -40276,12 +40444,12 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>Al Sidriya</t>
+          <t>Al Khbaib</t>
         </is>
       </c>
       <c r="D434" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478220</t>
+          <t>https://www.shipvault.com/ships/478217</t>
         </is>
       </c>
       <c r="E434" s="2" t="inlineStr">
@@ -40291,14 +40459,14 @@
       </c>
       <c r="F434" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2694 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2591 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069936 as AL KHBAIB</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>86</t>
         </is>
       </c>
       <c r="B435" s="2" t="inlineStr">
@@ -40308,12 +40476,12 @@
       </c>
       <c r="C435" s="2" t="inlineStr">
         <is>
-          <t>Al Sidriya</t>
+          <t>Al Khbaib</t>
         </is>
       </c>
       <c r="D435" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478220</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478217</t>
         </is>
       </c>
       <c r="E435" s="2" t="inlineStr">
@@ -40323,14 +40491,14 @@
       </c>
       <c r="F435" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2694 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2591 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069936 as AL KHBAIB</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>86</t>
         </is>
       </c>
       <c r="B436" s="2" t="inlineStr">
@@ -40340,29 +40508,29 @@
       </c>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>Lekhraib</t>
+          <t>Al Khbaib</t>
         </is>
       </c>
       <c r="D436" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/479139</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-KHBAIB/1069936/1</t>
         </is>
       </c>
       <c r="E436" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F436" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2694 (SHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2591 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069936 as AL KHBAIB</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>88</t>
         </is>
       </c>
       <c r="B437" s="2" t="inlineStr">
@@ -40372,29 +40540,29 @@
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>Lekhraib</t>
+          <t>Khowzan</t>
         </is>
       </c>
       <c r="D437" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479139</t>
+          <t>https://www.shipvault.com/ships/478218</t>
         </is>
       </c>
       <c r="E437" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F437" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2694 (SHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2592 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069948 as KHOWZAN</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>88</t>
         </is>
       </c>
       <c r="B438" s="2" t="inlineStr">
@@ -40404,29 +40572,29 @@
       </c>
       <c r="C438" s="2" t="inlineStr">
         <is>
-          <t>Ain Snan</t>
+          <t>Khowzan</t>
         </is>
       </c>
       <c r="D438" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478221</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478218</t>
         </is>
       </c>
       <c r="E438" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F438" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2695 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2592 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069948 as KHOWZAN</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>88</t>
         </is>
       </c>
       <c r="B439" s="2" t="inlineStr">
@@ -40436,29 +40604,29 @@
       </c>
       <c r="C439" s="2" t="inlineStr">
         <is>
-          <t>Ain Snan</t>
+          <t>Khowzan</t>
         </is>
       </c>
       <c r="D439" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478221</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/KHOWZAN/1069948/1</t>
         </is>
       </c>
       <c r="E439" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F439" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2695 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2592 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069948 as KHOWZAN</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>136</t>
         </is>
       </c>
       <c r="B440" s="2" t="inlineStr">
@@ -40468,12 +40636,12 @@
       </c>
       <c r="C440" s="2" t="inlineStr">
         <is>
-          <t>Al Wasmi</t>
+          <t>Al Ghafat</t>
         </is>
       </c>
       <c r="D440" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478222</t>
+          <t>https://www.shipvault.com/ships/478219</t>
         </is>
       </c>
       <c r="E440" s="2" t="inlineStr">
@@ -40483,14 +40651,14 @@
       </c>
       <c r="F440" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2696 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2693 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069950 as AL GHAFAT</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>136</t>
         </is>
       </c>
       <c r="B441" s="2" t="inlineStr">
@@ -40500,12 +40668,12 @@
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
-          <t>Al Wasmi</t>
+          <t>Al Ghafat</t>
         </is>
       </c>
       <c r="D441" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478222</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478219</t>
         </is>
       </c>
       <c r="E441" s="2" t="inlineStr">
@@ -40515,14 +40683,14 @@
       </c>
       <c r="F441" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2696 (Hanwha)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2693 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069950 as AL GHAFAT</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>136</t>
         </is>
       </c>
       <c r="B442" s="2" t="inlineStr">
@@ -40532,29 +40700,29 @@
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>Wadi Al Askar</t>
+          <t>Al Ghafat</t>
         </is>
       </c>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/479141</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-GHAFAT/1069950/1</t>
         </is>
       </c>
       <c r="E442" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F442" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2696 (SHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2693 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069950 as AL GHAFAT</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>138</t>
         </is>
       </c>
       <c r="B443" s="2" t="inlineStr">
@@ -40564,29 +40732,29 @@
       </c>
       <c r="C443" s="2" t="inlineStr">
         <is>
-          <t>Wadi Al Askar</t>
+          <t>Al Sidriya</t>
         </is>
       </c>
       <c r="D443" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479141</t>
+          <t>https://www.shipvault.com/ships/478220</t>
         </is>
       </c>
       <c r="E443" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F443" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2696 (SHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2694 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069962 as AL SIDRIYA</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>138</t>
         </is>
       </c>
       <c r="B444" s="2" t="inlineStr">
@@ -40596,29 +40764,29 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>Al Shaheen</t>
+          <t>Al Sidriya</t>
         </is>
       </c>
       <c r="D444" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/479144</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478220</t>
         </is>
       </c>
       <c r="E444" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F444" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2699 (SHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2694 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069962 as AL SIDRIYA</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>138</t>
         </is>
       </c>
       <c r="B445" s="2" t="inlineStr">
@@ -40628,29 +40796,29 @@
       </c>
       <c r="C445" s="2" t="inlineStr">
         <is>
-          <t>Al Shaheen</t>
+          <t>Al Sidriya</t>
         </is>
       </c>
       <c r="D445" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479144</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-SIDRIYA/1069962/1</t>
         </is>
       </c>
       <c r="E445" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F445" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2699 (SHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2694 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069962 as AL SIDRIYA</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>139</t>
         </is>
       </c>
       <c r="B446" s="2" t="inlineStr">
@@ -40660,12 +40828,12 @@
       </c>
       <c r="C446" s="2" t="inlineStr">
         <is>
-          <t>Al Nouf</t>
+          <t>Lekhraib</t>
         </is>
       </c>
       <c r="D446" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/479151</t>
+          <t>https://www.shipvault.com/ships/479139</t>
         </is>
       </c>
       <c r="E446" s="2" t="inlineStr">
@@ -40675,14 +40843,14 @@
       </c>
       <c r="F446" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2706 (SHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2694 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070727 as LEKHRAIB (MMSI 477262100)</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>139</t>
         </is>
       </c>
       <c r="B447" s="2" t="inlineStr">
@@ -40692,12 +40860,12 @@
       </c>
       <c r="C447" s="2" t="inlineStr">
         <is>
-          <t>Al Nouf</t>
+          <t>Lekhraib</t>
         </is>
       </c>
       <c r="D447" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479151</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479139</t>
         </is>
       </c>
       <c r="E447" s="2" t="inlineStr">
@@ -40707,14 +40875,14 @@
       </c>
       <c r="F447" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 2706 (SHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2694 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070727 as LEKHRAIB (MMSI 477262100)</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>139</t>
         </is>
       </c>
       <c r="B448" s="2" t="inlineStr">
@@ -40724,29 +40892,29 @@
       </c>
       <c r="C448" s="2" t="inlineStr">
         <is>
-          <t>Izghawa</t>
+          <t>Lekhraib</t>
         </is>
       </c>
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478320</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/LEKHRAIB/1070727/477262100</t>
         </is>
       </c>
       <c r="E448" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F448" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 3491 (HDHHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2694 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070727 as LEKHRAIB (MMSI 477262100)</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>140</t>
         </is>
       </c>
       <c r="B449" s="2" t="inlineStr">
@@ -40756,29 +40924,29 @@
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
-          <t>Izghawa</t>
+          <t>Ain Snan</t>
         </is>
       </c>
       <c r="D449" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478320</t>
+          <t>https://www.shipvault.com/ships/478221</t>
         </is>
       </c>
       <c r="E449" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F449" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 3491 (HDHHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2695 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069974 as AIN SNAN</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>140</t>
         </is>
       </c>
       <c r="B450" s="2" t="inlineStr">
@@ -40788,29 +40956,29 @@
       </c>
       <c r="C450" s="2" t="inlineStr">
         <is>
-          <t>Al Wa'ab</t>
+          <t>Ain Snan</t>
         </is>
       </c>
       <c r="D450" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/478321</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478221</t>
         </is>
       </c>
       <c r="E450" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F450" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 3492 (HDHHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2695 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069974 as AIN SNAN</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>140</t>
         </is>
       </c>
       <c r="B451" s="2" t="inlineStr">
@@ -40820,29 +40988,29 @@
       </c>
       <c r="C451" s="2" t="inlineStr">
         <is>
-          <t>Al Wa'ab</t>
+          <t>Ain Snan</t>
         </is>
       </c>
       <c r="D451" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478321</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AIN-SNAN/1069974/1</t>
         </is>
       </c>
       <c r="E451" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F451" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Hull 3492 (HDHHI)' -&gt; vessel named</t>
+          <t>placeholder 'Hull 2695 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069974 as AIN SNAN</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
         <is>
-          <t>508</t>
+          <t>142</t>
         </is>
       </c>
       <c r="B452" s="2" t="inlineStr">
@@ -40852,29 +41020,29 @@
       </c>
       <c r="C452" s="2" t="inlineStr">
         <is>
-          <t>Prime Glory</t>
+          <t>Al Wasmi</t>
         </is>
       </c>
       <c r="D452" s="2" t="inlineStr">
         <is>
-          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/PRIME-GLORY/1069194/1</t>
+          <t>https://www.shipvault.com/ships/478222</t>
         </is>
       </c>
       <c r="E452" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_clearance))</t>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
         </is>
       </c>
       <c r="F452" s="2" t="inlineStr">
         <is>
-          <t>placeholder 'Dalian No 1 G175K-11' -&gt; vessel named; marinetraffic.org lists IMO 1069194 as PRIME GLORY; shipvault still carries a hull placeholder - single source</t>
+          <t>placeholder 'Hull 2696 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069986 as AL WASMI</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>142</t>
         </is>
       </c>
       <c r="B453" s="2" t="inlineStr">
@@ -40884,29 +41052,29 @@
       </c>
       <c r="C453" s="2" t="inlineStr">
         <is>
-          <t>Friendship Venture</t>
+          <t>Al Wasmi</t>
         </is>
       </c>
       <c r="D453" s="2" t="inlineStr">
         <is>
-          <t>https://www.shipvault.com/ships/469427</t>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478222</t>
         </is>
       </c>
       <c r="E453" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+          <t>PASS (OK (shipvault_api))</t>
         </is>
       </c>
       <c r="F453" s="2" t="inlineStr">
         <is>
-          <t>backend 'Dalian No 1 G175K-12' differs from registry name; marinetraffic.org independently lists IMO 1030557 as FRIENDSHIP VENTURE (MMSI 636025371)</t>
+          <t>placeholder 'Hull 2696 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069986 as AL WASMI</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>142</t>
         </is>
       </c>
       <c r="B454" s="2" t="inlineStr">
@@ -40916,52 +41084,660 @@
       </c>
       <c r="C454" s="2" t="inlineStr">
         <is>
-          <t>Friendship Venture</t>
+          <t>Al Wasmi</t>
         </is>
       </c>
       <c r="D454" s="2" t="inlineStr">
         <is>
-          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/469427</t>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-WASMI/1069986/1</t>
         </is>
       </c>
       <c r="E454" s="2" t="inlineStr">
         <is>
-          <t>PASS (OK (shipvault_api))</t>
+          <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
       <c r="F454" s="2" t="inlineStr">
         <is>
-          <t>backend 'Dalian No 1 G175K-12' differs from registry name; marinetraffic.org independently lists IMO 1030557 as FRIENDSHIP VENTURE (MMSI 636025371)</t>
+          <t>placeholder 'Hull 2696 (Hanwha)' -&gt; vessel named; marinetraffic.org independently lists IMO 1069986 as AL WASMI</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
         <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="B455" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C455" s="2" t="inlineStr">
+        <is>
+          <t>Wadi Al Askar</t>
+        </is>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/479141</t>
+        </is>
+      </c>
+      <c r="E455" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2696 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070739 as WADI AL ASKAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="B456" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C456" s="2" t="inlineStr">
+        <is>
+          <t>Wadi Al Askar</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479141</t>
+        </is>
+      </c>
+      <c r="E456" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F456" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2696 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070739 as WADI AL ASKAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="inlineStr">
+        <is>
+          <t>143</t>
+        </is>
+      </c>
+      <c r="B457" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C457" s="2" t="inlineStr">
+        <is>
+          <t>Wadi Al Askar</t>
+        </is>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/WADI-AL-ASKAR/1070739/1</t>
+        </is>
+      </c>
+      <c r="E457" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_clearance))</t>
+        </is>
+      </c>
+      <c r="F457" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2696 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070739 as WADI AL ASKAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="B458" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C458" s="2" t="inlineStr">
+        <is>
+          <t>Al Shaheen</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/479144</t>
+        </is>
+      </c>
+      <c r="E458" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F458" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2699 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070741 as AL SHAHEEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="B459" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C459" s="2" t="inlineStr">
+        <is>
+          <t>Al Shaheen</t>
+        </is>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479144</t>
+        </is>
+      </c>
+      <c r="E459" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F459" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2699 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070741 as AL SHAHEEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>146</t>
+        </is>
+      </c>
+      <c r="B460" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C460" s="2" t="inlineStr">
+        <is>
+          <t>Al Shaheen</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-SHAHEEN/1070741/1</t>
+        </is>
+      </c>
+      <c r="E460" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_clearance))</t>
+        </is>
+      </c>
+      <c r="F460" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2699 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070741 as AL SHAHEEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="B461" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C461" s="2" t="inlineStr">
+        <is>
+          <t>Libsayer</t>
+        </is>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/LIBSAYER/1070806/1</t>
+        </is>
+      </c>
+      <c r="E461" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_clearance))</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2702 (SHI)' -&gt; vessel named; marinetraffic.org lists IMO 1070806 as LIBSAYER; shipvault still carries a hull placeholder - single source</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="B462" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C462" s="2" t="inlineStr">
+        <is>
+          <t>Al Nouf</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/479151</t>
+        </is>
+      </c>
+      <c r="E462" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2706 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070820 as AL NOUF</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="B463" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C463" s="2" t="inlineStr">
+        <is>
+          <t>Al Nouf</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/479151</t>
+        </is>
+      </c>
+      <c r="E463" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2706 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070820 as AL NOUF</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>154</t>
+        </is>
+      </c>
+      <c r="B464" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>Al Nouf</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-NOUF/1070820/1</t>
+        </is>
+      </c>
+      <c r="E464" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_clearance))</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 2706 (SHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1070820 as AL NOUF</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B465" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C465" s="2" t="inlineStr">
+        <is>
+          <t>Izghawa</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/478320</t>
+        </is>
+      </c>
+      <c r="E465" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 3491 (HDHHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1049091 as IZGHAWA</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B466" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>Izghawa</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478320</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 3491 (HDHHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1049091 as IZGHAWA</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B467" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C467" s="2" t="inlineStr">
+        <is>
+          <t>Izghawa</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/IZGHAWA/1049091/1</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_clearance))</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 3491 (HDHHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1049091 as IZGHAWA</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="B468" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C468" s="2" t="inlineStr">
+        <is>
+          <t>Al Wa'ab</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/478321</t>
+        </is>
+      </c>
+      <c r="E468" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 3492 (HDHHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1049118 as AL WA'AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="B469" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C469" s="2" t="inlineStr">
+        <is>
+          <t>Al Wa'ab</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/478321</t>
+        </is>
+      </c>
+      <c r="E469" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 3492 (HDHHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1049118 as AL WA'AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="B470" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C470" s="2" t="inlineStr">
+        <is>
+          <t>Al Wa'ab</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/AL-WA'AB/1049118/1</t>
+        </is>
+      </c>
+      <c r="E470" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_clearance))</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Hull 3492 (HDHHI)' -&gt; vessel named; marinetraffic.org independently lists IMO 1049118 as AL WA'AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="inlineStr">
+        <is>
+          <t>508</t>
+        </is>
+      </c>
+      <c r="B471" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C471" s="2" t="inlineStr">
+        <is>
+          <t>Prime Glory</t>
+        </is>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/PRIME-GLORY/1069194/1</t>
+        </is>
+      </c>
+      <c r="E471" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_clearance))</t>
+        </is>
+      </c>
+      <c r="F471" s="2" t="inlineStr">
+        <is>
+          <t>placeholder 'Dalian No 1 G175K-11' -&gt; vessel named; marinetraffic.org lists IMO 1069194 as PRIME GLORY; shipvault still carries a hull placeholder - single source</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
           <t>509</t>
         </is>
       </c>
-      <c r="B455" s="2" t="inlineStr">
+      <c r="B472" s="2" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C455" s="2" t="inlineStr">
+      <c r="C472" s="2" t="inlineStr">
         <is>
           <t>Friendship Venture</t>
         </is>
       </c>
-      <c r="D455" s="2" t="inlineStr">
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>https://www.shipvault.com/ships/469427</t>
+        </is>
+      </c>
+      <c r="E472" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (cf_impersonate, shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="inlineStr">
+        <is>
+          <t>backend 'Dalian No 1 G175K-12' differs from registry name; marinetraffic.org independently lists IMO 1030557 as FRIENDSHIP VENTURE (MMSI 636025371)</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="inlineStr">
+        <is>
+          <t>509</t>
+        </is>
+      </c>
+      <c r="B473" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C473" s="2" t="inlineStr">
+        <is>
+          <t>Friendship Venture</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>https://shipvaultapi-gjb8c.ondigitalocean.app/api/units/469427</t>
+        </is>
+      </c>
+      <c r="E473" s="2" t="inlineStr">
+        <is>
+          <t>PASS (OK (shipvault_api))</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="inlineStr">
+        <is>
+          <t>backend 'Dalian No 1 G175K-12' differs from registry name; marinetraffic.org independently lists IMO 1030557 as FRIENDSHIP VENTURE (MMSI 636025371)</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>509</t>
+        </is>
+      </c>
+      <c r="B474" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C474" s="2" t="inlineStr">
+        <is>
+          <t>Friendship Venture</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
         <is>
           <t>https://www.marinetraffic.org/ship-owner-manager-ism-data/FRIENDSHIP-VENTURE/1030557/636025371</t>
         </is>
       </c>
-      <c r="E455" s="2" t="inlineStr">
+      <c r="E474" s="2" t="inlineStr">
         <is>
           <t>PASS (OK (cf_clearance))</t>
         </is>
       </c>
-      <c r="F455" s="2" t="inlineStr">
+      <c r="F474" s="2" t="inlineStr">
         <is>
           <t>backend 'Dalian No 1 G175K-12' differs from registry name; marinetraffic.org independently lists IMO 1030557 as FRIENDSHIP VENTURE (MMSI 636025371)</t>
         </is>

</xml_diff>